<commit_message>
Champs requis pour l'invitation Spruce : nom complet, cellulaire (texto), courriel
- Registre : colonne « Cellulaire (texto) » + règle obligatoire dans les
  instructions (pour chaque personne, membre et famille)
- /arpq : les courriels d'inscription préremplis demandent le cellulaire
  pouvant recevoir des textos (FR/EN)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PwbBsCU7dC8TRedcQSdPwW
</commit_message>
<xml_diff>
--- a/arpq/registre-modele.xlsx
+++ b/arpq/registre-modele.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0 $"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,6 +92,12 @@
       <sz val="11"/>
     </font>
     <font/>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -158,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -192,6 +198,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -630,7 +639,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Téléphone</t>
+          <t>Cellulaire (texto)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -10296,7 +10305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -10337,130 +10346,142 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
+          <t>1b.</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>OBLIGATOIRE pour l'invitation Spruce — pour CHAQUE personne (membre ET famille) : prénom + nom, CELLULAIRE pouvant recevoir des textos, et courriel. Sans ces trois informations, pas d'invitation possible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Statut « Actif » dès que la personne est couverte par le paiement de l'ARPQ.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Quand une personne cesse d'être couverte (départ, non-paiement des cotisations) : Statut « Grâce 90 jours » + inscrire la Date de retrait. La colonne « Fin de grâce » se calcule seule.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Ne jamais effacer une ligne — passer le statut à « Retiré » après la grâce.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="20" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="20" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>CÔTÉ CLINIQUE (colonnes BLEU PÂLE)</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Règle d'or : aucun nom au registre payé = aucune invitation Spruce.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>6.</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Chaque jour : onglet Facturation, case « Invitations à faire » → envoyer l'invitation Spruce + le courriel modèle (brouillon Gmail « MODÈLE — Bienvenue ») → marquer Invité = Oui + date.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>7.</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>À la Fin de grâce : désactiver la personne dans Spruce, passer le statut à « Retiré ».</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>8.</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Chaque début de mois : figer les chiffres dans l'HISTORIQUE (onglet Facturation) et envoyer la facture Stripe à l'ARPQ (personnes actives × tarif).</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="20" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="20" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>PARTAGE</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>9.</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Une fois converti en Google Sheet : Partager → cff@centremedicalfont.ca (Éditeur) + la personne-ressource ARPQ (Éditeur). Personne d'autre.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>10.</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Les données de santé ne vont JAMAIS dans ce fichier — seulement l'identité et les coordonnées (Loi 25 : minimisation).</t>
         </is>

</xml_diff>

<commit_message>
Paliers: bloc banque de consultations gratuites sur accueil, tsq, entreprises, hedhofis
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8ao8kQtd2348jDRjtEdaK
</commit_message>
<xml_diff>
--- a/arpq/registre-modele.xlsx
+++ b/arpq/registre-modele.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos Faviel Font\truckstopsante-site\arpq\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BA4CF8-E3A9-4761-8D4E-805DF6CE9DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8BDF3C-38B0-4BE8-87AC-AA2677C1EB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="93">
   <si>
     <t>TRUCK STOP SANTÉ × ARPQ — REGISTRE DES PERSONNES COUVERTES</t>
   </si>
@@ -263,31 +263,13 @@
     <t>Les données de santé ne vont JAMAIS dans ce fichier — seulement l'identité et les coordonnées (Loi 25 : minimisation).</t>
   </si>
   <si>
-    <t>BANQUE DE CONSULTATIONS GRATUITES - POUR QUI l'ARPQ VEUT (pas besoin de payer, envoyez-les-nous)</t>
-  </si>
-  <si>
     <t>Personnes ACTIVES au registre (en direct) :</t>
-  </si>
-  <si>
-    <t>Règle : 5 consultations gratuites par mois par tranche de 100 personnes couvertes (1 000 = 50)</t>
   </si>
   <si>
     <t>CONSULTATIONS GRATUITES DISPONIBLES CE MOIS :</t>
   </si>
   <si>
-    <t>Utilisées ce mois (compte automatique des lignes du mois courant) :</t>
-  </si>
-  <si>
     <t>Restantes ce mois :</t>
-  </si>
-  <si>
-    <t>Date d'envoi</t>
-  </si>
-  <si>
-    <t>Envoyé par (ARPQ / entreprise)</t>
-  </si>
-  <si>
-    <t>Invité Spruce le</t>
   </si>
   <si>
     <t>Notes (jamais de données de santé)</t>
@@ -305,10 +287,34 @@
     <t>marc@exemple.com</t>
   </si>
   <si>
-    <t>Steve B.</t>
+    <t>EXEMPLE - supprimer cette ligne</t>
   </si>
   <si>
-    <t>EXEMPLE - supprimer cette ligne</t>
+    <t>BANQUE DE CONSULTATIONS GRATUITES - 1 ligne = 1 consultation - avec le code de l'ARPQ - famille et non-inscrits, sans abonnement</t>
+  </si>
+  <si>
+    <t>Règle : 5 consultations gratuites par mois par tranche de 100 personnes couvertes (1 000 = 50). Renouvelée chaque mois, NON cumulable. Quelqu'un qui a besoin de 5 consultations dans le mois en utilise 5.</t>
+  </si>
+  <si>
+    <t>CODE À DONNER :</t>
+  </si>
+  <si>
+    <t>ARPQ-SANTE</t>
+  </si>
+  <si>
+    <t>Consultations utilisées ce mois (compte automatique des lignes du mois courant) :</t>
+  </si>
+  <si>
+    <t>Date de la consultation</t>
+  </si>
+  <si>
+    <t>Code utilisé</t>
+  </si>
+  <si>
+    <t>Lien avec un membre (famille / non-inscrit)</t>
+  </si>
+  <si>
+    <t>conjoint de J. Tremblay</t>
   </si>
 </sst>
 </file>
@@ -534,6 +540,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -545,12 +557,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -872,44 +878,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
     </row>
     <row r="3" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -10203,15 +10209,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
@@ -10525,10 +10531,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="21"/>
+      <c r="B1" s="27"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
@@ -10672,20 +10678,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A1" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
+      <c r="A1" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B3">
         <f>Facturation!B5</f>
@@ -10694,21 +10708,21 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="28">
+      <c r="A5" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="21">
         <f>INT(B3/100)*5</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B6">
         <f ca="1">COUNTIFS(A10:A509,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),A10:A509,"&lt;"&amp;DATE(YEAR(TODAY()),MONTH(TODAY())+1,1))</f>
@@ -10716,61 +10730,64 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="27">
+      <c r="A7" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="20">
         <f ca="1">B5-B6</f>
         <v>-1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" s="22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="23">
+        <v>46280</v>
+      </c>
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="29" t="s">
+      <c r="E10" t="s">
         <v>82</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="F10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" t="s">
         <v>83</v>
-      </c>
-      <c r="H9" s="29" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="30">
-        <v>46280</v>
-      </c>
-      <c r="B10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" t="s">
-        <v>86</v>
-      </c>
-      <c r="D10" t="s">
-        <v>87</v>
-      </c>
-      <c r="E10" t="s">
-        <v>88</v>
-      </c>
-      <c r="F10" t="s">
-        <v>89</v>
-      </c>
-      <c r="H10" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>